<commit_message>
cambios esquema user y excel
</commit_message>
<xml_diff>
--- a/src/shared/reportes.xlsx
+++ b/src/shared/reportes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andres\tarificador\Transfer-Call-Demo-Backend\src\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3087ACCE-8ED6-4EE5-9768-FFFFEB0F5C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF4FBFF-A08D-4227-A7E8-B2AC678E9756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5085" yWindow="765" windowWidth="21600" windowHeight="9810" firstSheet="1" activeTab="4" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
+    <workbookView xWindow="3300" yWindow="3030" windowWidth="21600" windowHeight="9810" firstSheet="2" activeTab="7" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
   </bookViews>
   <sheets>
     <sheet name="generalEntidad1" sheetId="8" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="adminGeneralReporte" sheetId="5" r:id="rId5"/>
     <sheet name="sede1" sheetId="3" r:id="rId6"/>
     <sheet name="sede2" sheetId="4" r:id="rId7"/>
+    <sheet name="11235648542" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="101">
   <si>
     <t>Llamada</t>
   </si>
@@ -333,6 +334,18 @@
   </si>
   <si>
     <t>larga distancia inter</t>
+  </si>
+  <si>
+    <t>Numero</t>
+  </si>
+  <si>
+    <t>Cant llamadas</t>
+  </si>
+  <si>
+    <t>Cant minutos</t>
+  </si>
+  <si>
+    <t>Cobro total</t>
   </si>
 </sst>
 </file>
@@ -451,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -503,6 +516,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2564,4 +2578,59 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7807B4AD-F5DA-4CD1-B499-3CC170EFFF63}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2">
+        <v>18682207777</v>
+      </c>
+      <c r="C2">
+        <v>6</v>
+      </c>
+      <c r="D2" s="23">
+        <v>1.5277777777777777E-2</v>
+      </c>
+      <c r="E2">
+        <v>19.8</v>
+      </c>
+      <c r="G2">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C3" s="22"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Cambios reportes y modulo usuario
</commit_message>
<xml_diff>
--- a/src/shared/reportes.xlsx
+++ b/src/shared/reportes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andres\tarificador\Transfer-Call-Demo-Backend\src\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF4FBFF-A08D-4227-A7E8-B2AC678E9756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91041C26-3378-4597-8D35-A2692FA7EA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="3030" windowWidth="21600" windowHeight="9810" firstSheet="2" activeTab="7" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="7" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
   </bookViews>
   <sheets>
     <sheet name="generalEntidad1" sheetId="8" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="adminGeneralReporte" sheetId="5" r:id="rId5"/>
     <sheet name="sede1" sheetId="3" r:id="rId6"/>
     <sheet name="sede2" sheetId="4" r:id="rId7"/>
-    <sheet name="11235648542" sheetId="10" r:id="rId8"/>
+    <sheet name="number" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="104">
   <si>
     <t>Llamada</t>
   </si>
@@ -346,6 +346,15 @@
   </si>
   <si>
     <t>Cobro total</t>
+  </si>
+  <si>
+    <t>Fecha inicio</t>
+  </si>
+  <si>
+    <t>Fecha final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entidad2 </t>
   </si>
 </sst>
 </file>
@@ -464,7 +473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -517,6 +526,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2582,12 +2593,15 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7807B4AD-F5DA-4CD1-B499-3CC170EFFF63}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
     <col min="3" max="3" width="22.42578125" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2606,6 +2620,12 @@
       <c r="E1" t="s">
         <v>100</v>
       </c>
+      <c r="F1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G1" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -2623,12 +2643,127 @@
       <c r="E2">
         <v>19.8</v>
       </c>
-      <c r="G2">
-        <v>0.9</v>
+      <c r="F2" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G2" s="24">
+        <v>45806.625</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C3" s="22"/>
+      <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3">
+        <v>12365987634</v>
+      </c>
+      <c r="C3" s="25">
+        <v>5</v>
+      </c>
+      <c r="D3" s="23">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="E3">
+        <v>11.7</v>
+      </c>
+      <c r="F3" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G3" s="24">
+        <v>45806.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4">
+        <v>59875642351</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="23">
+        <v>5.5555555555555558E-3</v>
+      </c>
+      <c r="E4">
+        <v>9.5</v>
+      </c>
+      <c r="F4" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G4" s="24">
+        <v>45806.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5">
+        <v>36987752154</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5" s="23">
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="E5">
+        <v>22.5</v>
+      </c>
+      <c r="F5" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G5" s="24">
+        <v>45806.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6">
+        <v>89653251126</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" s="23">
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="E6">
+        <v>13.5</v>
+      </c>
+      <c r="F6" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G6" s="24">
+        <v>45806.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7">
+        <v>86523689856</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" s="23">
+        <v>6.2500000000000003E-3</v>
+      </c>
+      <c r="E7">
+        <v>10.5</v>
+      </c>
+      <c r="F7" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G7" s="24">
+        <v>45806.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambios envio de correos y tarificador
</commit_message>
<xml_diff>
--- a/src/shared/reportes.xlsx
+++ b/src/shared/reportes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andres\tarificador\Transfer-Call-Demo-Backend\src\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7932172C-922F-4946-8337-AA99827BE797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2A995C-170D-4BB1-9E95-7F9D6D847755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2385" yWindow="2235" windowWidth="25950" windowHeight="12000" activeTab="4" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="2" activeTab="2" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
   </bookViews>
   <sheets>
     <sheet name="generalEntidad1" sheetId="8" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="117">
   <si>
     <t>Llamada</t>
   </si>
@@ -2670,7 +2670,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7807B4AD-F5DA-4CD1-B499-3CC170EFFF63}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -2715,10 +2715,11 @@
         <v>6</v>
       </c>
       <c r="D2" s="23">
-        <v>1.5277777777777777E-2</v>
+        <v>3.0555555555555555E-2</v>
       </c>
       <c r="E2">
-        <v>19.8</v>
+        <f>19.8*2</f>
+        <v>39.6</v>
       </c>
       <c r="F2" s="24">
         <v>45778.333333333336</v>
@@ -2732,16 +2733,16 @@
         <v>89</v>
       </c>
       <c r="B3">
-        <v>12365987634</v>
+        <v>54697584352</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3" s="23">
-        <v>1.0416666666666666E-2</v>
+        <v>4.8611111111111112E-3</v>
       </c>
       <c r="E3">
-        <v>11.7</v>
+        <v>7</v>
       </c>
       <c r="F3" s="24">
         <v>45778.333333333336</v>
@@ -2755,39 +2756,39 @@
         <v>89</v>
       </c>
       <c r="B4">
-        <v>59875642351</v>
+        <v>85469757431</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="23">
-        <v>5.5555555555555558E-3</v>
+        <v>1.3888888888888889E-3</v>
       </c>
       <c r="E4">
-        <v>9.5</v>
+        <v>2</v>
       </c>
       <c r="F4" s="24">
         <v>45778.333333333336</v>
       </c>
       <c r="G4" s="24">
-        <v>45806.5</v>
+        <v>45807.5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5">
-        <v>36987752154</v>
+        <v>65469758430</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D5" s="23">
-        <v>1.6666666666666666E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="E5">
-        <v>22.5</v>
+        <v>10</v>
       </c>
       <c r="F5" s="24">
         <v>45778.333333333336</v>
@@ -2801,16 +2802,16 @@
         <v>90</v>
       </c>
       <c r="B6">
-        <v>89653251126</v>
+        <v>82469758470</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D6" s="23">
-        <v>1.2500000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="F6" s="24">
         <v>45778.333333333336</v>
@@ -2824,16 +2825,16 @@
         <v>90</v>
       </c>
       <c r="B7">
-        <v>86523689856</v>
+        <v>85009758430</v>
       </c>
       <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" s="23">
+        <v>2.0833333333333333E-3</v>
+      </c>
+      <c r="E7">
         <v>3</v>
-      </c>
-      <c r="D7" s="23">
-        <v>6.2500000000000003E-3</v>
-      </c>
-      <c r="E7">
-        <v>10.5</v>
       </c>
       <c r="F7" s="24">
         <v>45778.333333333336</v>
@@ -2842,7 +2843,54 @@
         <v>45806.5</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8">
+        <v>56469758420</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="23">
+        <v>2.7777777777777779E-3</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G8" s="24">
+        <v>45806.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9">
+        <v>85469758430</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" s="23">
+        <v>7.6388888888888886E-3</v>
+      </c>
+      <c r="E9">
+        <v>11</v>
+      </c>
+      <c r="F9" s="24">
+        <v>45778.333333333336</v>
+      </c>
+      <c r="G9" s="24">
+        <v>45807.5</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cambios reporte general excel
</commit_message>
<xml_diff>
--- a/src/shared/reportes.xlsx
+++ b/src/shared/reportes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andres\tarificador\Transfer-Call-Demo-Backend\src\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2A995C-170D-4BB1-9E95-7F9D6D847755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CC9C4A-8C22-4473-B818-1FD05037034F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="2" activeTab="2" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="25950" windowHeight="12000" firstSheet="2" activeTab="4" xr2:uid="{BBF53177-29A7-4A37-87D8-7C5D15F0C2A9}"/>
   </bookViews>
   <sheets>
     <sheet name="generalEntidad1" sheetId="8" r:id="rId1"/>
@@ -401,6 +401,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -518,7 +521,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -567,6 +569,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -946,10 +949,10 @@
       <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -982,15 +985,15 @@
       <c r="I2">
         <v>31.55</v>
       </c>
-      <c r="J2" s="24">
+      <c r="J2" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="K2" s="24">
+      <c r="K2" s="23">
         <v>45806.625</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I13" s="22"/>
+      <c r="I13" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1168,10 +1171,10 @@
       <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1204,10 +1207,10 @@
       <c r="I2">
         <v>39.049999999999997</v>
       </c>
-      <c r="J2" s="24">
+      <c r="J2" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="K2" s="24">
+      <c r="K2" s="23">
         <v>45806.625</v>
       </c>
     </row>
@@ -1354,44 +1357,44 @@
     <col min="13" max="13" width="22.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1427,7 +1430,7 @@
         <f>generalEntidad11!C2+generalEntidad11!C3+generalEntidad11!C4+generalEntidad11!C5+generalEntidad11!C6</f>
         <v>80</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="24">
         <f>generalEntidad11!E2+generalEntidad11!E3+generalEntidad11!E4+generalEntidad11!E5+generalEntidad11!E6</f>
         <v>31.549999999999997</v>
       </c>
@@ -1437,10 +1440,10 @@
       <c r="K2" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="24">
+      <c r="L2" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="M2" s="24">
+      <c r="M2" s="23">
         <v>45806.625</v>
       </c>
     </row>
@@ -1476,7 +1479,7 @@
         <f>SUM(generalEntidad22!C2:C6)</f>
         <v>100</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="24">
         <f>SUM(generalEntidad22!E2:E6)</f>
         <v>39.049999999999997</v>
       </c>
@@ -1486,10 +1489,10 @@
       <c r="K3" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="24">
+      <c r="L3" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="M3" s="24">
+      <c r="M3" s="23">
         <v>45806.625</v>
       </c>
     </row>
@@ -1497,7 +1500,7 @@
       <c r="A4" s="1"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H8" s="22"/>
+      <c r="H8" s="21"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1511,612 +1514,612 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="6" customWidth="1"/>
-    <col min="4" max="4" width="26.42578125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.5703125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="6"/>
-    <col min="7" max="7" width="13.28515625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="6"/>
+    <col min="1" max="1" width="25.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="26.42578125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="5"/>
+    <col min="7" max="7" width="13.28515625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>5.6712962962962967E-3</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="9">
         <v>9</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="10">
         <v>0.25</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="10">
         <f t="shared" ref="I2:I20" si="0">G2*H2</f>
         <v>2.25</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="8">
         <v>1.7592592592592592E-3</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>3</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>0.5</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="8">
         <v>3.8657407407407408E-3</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>6</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>0.5</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="8">
         <v>3.9236111111111112E-3</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <v>6</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <v>0.35</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <f t="shared" si="0"/>
         <v>2.0999999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="8">
         <v>2.685185185185185E-3</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <v>4</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>0.5</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="8">
         <v>4.5138888888888885E-3</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="9">
         <v>7</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <v>0.5</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="10">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="9">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10">
-        <v>0</v>
-      </c>
-      <c r="H8" s="11">
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10">
         <v>0.25</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="8">
         <v>3.2407407407407406E-3</v>
       </c>
-      <c r="G9" s="10">
-        <v>5</v>
-      </c>
-      <c r="H9" s="11">
+      <c r="G9" s="9">
+        <v>5</v>
+      </c>
+      <c r="H9" s="10">
         <v>0.25</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="10">
         <f t="shared" si="0"/>
         <v>1.25</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="8">
         <v>1.7013888888888888E-3</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="9">
         <v>3</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <v>0.35</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="10">
         <f t="shared" si="0"/>
         <v>1.0499999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="8">
         <v>3.5879629629629629E-3</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="9">
         <v>6</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="10">
         <v>0.25</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="10">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="9">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10">
-        <v>0</v>
-      </c>
-      <c r="H12" s="11">
+      <c r="F12" s="8">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10">
         <v>0.25</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="8">
         <v>4.6064814814814814E-3</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="9">
         <v>7</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="10">
         <v>0.25</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <f t="shared" si="0"/>
         <v>1.75</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="8">
         <v>2.6041666666666665E-3</v>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="9">
         <v>4</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <v>0.25</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="10">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="9">
-        <v>0</v>
-      </c>
-      <c r="G15" s="10">
-        <v>0</v>
-      </c>
-      <c r="H15" s="11">
+      <c r="F15" s="8">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10">
         <v>0.5</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="8">
         <v>6.0185185185185185E-3</v>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="9">
         <v>9</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="10">
         <v>0.5</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="10">
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="8" t="s">
+      <c r="A17" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="8">
         <v>3.8194444444444443E-3</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="9">
         <v>6</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="10">
         <v>0.25</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="10">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="8">
         <v>3.1250000000000002E-3</v>
       </c>
-      <c r="G18" s="12">
-        <v>5</v>
-      </c>
-      <c r="H18" s="11">
+      <c r="G18" s="11">
+        <v>5</v>
+      </c>
+      <c r="H18" s="10">
         <v>0.5</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="10">
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F19" s="9">
-        <v>0</v>
-      </c>
-      <c r="G19" s="12">
-        <v>0</v>
-      </c>
-      <c r="H19" s="13">
+      <c r="F19" s="8">
+        <v>0</v>
+      </c>
+      <c r="G19" s="11">
+        <v>0</v>
+      </c>
+      <c r="H19" s="12">
         <v>0.5</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="9">
-        <v>0</v>
-      </c>
-      <c r="G20" s="14">
-        <v>0</v>
-      </c>
-      <c r="H20" s="15">
+      <c r="F20" s="8">
+        <v>0</v>
+      </c>
+      <c r="G20" s="13">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14">
         <v>0.5</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2143,520 +2146,520 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="17" t="s">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="17" t="s">
         <v>4</v>
       </c>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="18" t="s">
+      <c r="A2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="18">
         <v>6.9444444444444441E-3</v>
       </c>
-      <c r="G2" s="20">
+      <c r="G2" s="19">
         <v>10</v>
       </c>
-      <c r="H2" s="18">
+      <c r="H2" s="17">
         <v>0.25</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="17">
         <f t="shared" ref="I2:I17" si="0">G2*H2</f>
         <v>2.5</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="18">
         <v>6.5972222222222222E-3</v>
       </c>
-      <c r="G3" s="20">
+      <c r="G3" s="19">
         <v>10</v>
       </c>
-      <c r="H3" s="18">
+      <c r="H3" s="17">
         <v>0.5</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="17">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="18">
         <v>5.7870370370370367E-3</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="19">
         <v>9</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="17">
         <v>0.5</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="17">
         <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="18">
         <v>4.1666666666666666E-3</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="19">
         <v>6</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="17">
         <v>0.35</v>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="17">
         <f t="shared" si="0"/>
         <v>2.0999999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="18">
         <v>8.3333333333333332E-3</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <v>12</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="17">
         <v>0.6</v>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="17">
         <f t="shared" si="0"/>
         <v>7.1999999999999993</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="18">
         <v>4.5138888888888885E-3</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="19">
         <v>7</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="17">
         <v>0.5</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="17">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="18" t="s">
+      <c r="A8" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="19">
-        <v>0</v>
-      </c>
-      <c r="G8" s="20">
-        <v>0</v>
-      </c>
-      <c r="H8" s="18">
+      <c r="F8" s="18">
+        <v>0</v>
+      </c>
+      <c r="G8" s="19">
+        <v>0</v>
+      </c>
+      <c r="H8" s="17">
         <v>0.25</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="18" t="s">
+      <c r="A9" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="F9" s="19">
-        <v>0</v>
-      </c>
-      <c r="G9" s="20">
-        <v>0</v>
-      </c>
-      <c r="H9" s="18">
+      <c r="F9" s="18">
+        <v>0</v>
+      </c>
+      <c r="G9" s="19">
+        <v>0</v>
+      </c>
+      <c r="H9" s="17">
         <v>0.25</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="18" t="s">
+      <c r="A10" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="18">
         <v>1.3888888888888888E-2</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="19">
         <v>20</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="17">
         <v>0.25</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="17">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="18" t="s">
+      <c r="A11" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="19">
-        <v>0</v>
-      </c>
-      <c r="G11" s="21">
-        <v>0</v>
-      </c>
-      <c r="H11" s="18">
+      <c r="F11" s="18">
+        <v>0</v>
+      </c>
+      <c r="G11" s="20">
+        <v>0</v>
+      </c>
+      <c r="H11" s="17">
         <v>0.25</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="18">
         <v>5.092592592592593E-3</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="19">
         <v>8</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="17">
         <v>0.5</v>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="17">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="18" t="s">
+      <c r="A13" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="18">
         <v>3.1250000000000002E-3</v>
       </c>
-      <c r="G13" s="20">
-        <v>5</v>
-      </c>
-      <c r="H13" s="18">
+      <c r="G13" s="19">
+        <v>5</v>
+      </c>
+      <c r="H13" s="17">
         <v>0.25</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="17">
         <f t="shared" si="0"/>
         <v>1.25</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="19">
-        <v>0</v>
-      </c>
-      <c r="G14" s="20">
-        <v>0</v>
-      </c>
-      <c r="H14" s="18">
+      <c r="F14" s="18">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19">
+        <v>0</v>
+      </c>
+      <c r="H14" s="17">
         <v>0.5</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="18">
         <v>3.7037037037037038E-3</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="20">
         <v>6</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="17">
         <v>0.5</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="17">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="18" t="s">
+      <c r="A16" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="18">
         <v>3.472222222222222E-3</v>
       </c>
-      <c r="G16" s="20">
-        <v>5</v>
-      </c>
-      <c r="H16" s="18">
+      <c r="G16" s="19">
+        <v>5</v>
+      </c>
+      <c r="H16" s="17">
         <v>0.25</v>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="17">
         <f t="shared" si="0"/>
         <v>1.25</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="18" t="s">
+      <c r="A17" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="18">
         <v>3.8194444444444443E-3</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <v>6</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="17">
         <v>0.25</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="17">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F18" s="5"/>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F19" s="5"/>
+      <c r="F19" s="4"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -2714,17 +2717,17 @@
       <c r="C2">
         <v>6</v>
       </c>
-      <c r="D2" s="23">
+      <c r="D2" s="22">
         <v>3.0555555555555555E-2</v>
       </c>
       <c r="E2">
         <f>19.8*2</f>
         <v>39.6</v>
       </c>
-      <c r="F2" s="24">
+      <c r="F2" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G2" s="24">
+      <c r="G2" s="23">
         <v>45806.625</v>
       </c>
     </row>
@@ -2738,16 +2741,16 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3" s="23">
+      <c r="D3" s="22">
         <v>4.8611111111111112E-3</v>
       </c>
       <c r="E3">
         <v>7</v>
       </c>
-      <c r="F3" s="24">
+      <c r="F3" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G3" s="24">
+      <c r="G3" s="23">
         <v>45806.5</v>
       </c>
     </row>
@@ -2761,16 +2764,16 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="22">
         <v>1.3888888888888889E-3</v>
       </c>
       <c r="E4">
         <v>2</v>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="23">
         <v>45807.5</v>
       </c>
     </row>
@@ -2784,16 +2787,16 @@
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="22">
         <v>6.9444444444444441E-3</v>
       </c>
       <c r="E5">
         <v>10</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="23">
         <v>45806.5</v>
       </c>
     </row>
@@ -2807,16 +2810,16 @@
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="22">
         <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="23">
         <v>45806.5</v>
       </c>
     </row>
@@ -2830,16 +2833,16 @@
       <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <v>2.0833333333333333E-3</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="23">
         <v>45806.5</v>
       </c>
     </row>
@@ -2853,16 +2856,16 @@
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="22">
         <v>2.7777777777777779E-3</v>
       </c>
       <c r="E8">
         <v>4</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="23">
         <v>45806.5</v>
       </c>
     </row>
@@ -2876,16 +2879,16 @@
       <c r="C9">
         <v>2</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <v>7.6388888888888886E-3</v>
       </c>
       <c r="E9">
         <v>11</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="23">
         <v>45778.333333333336</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="23">
         <v>45807.5</v>
       </c>
     </row>

</xml_diff>